<commit_message>
bob 执行su - bob -c 'docker network connect alice-net $(docker run -d nginx:alpine)' 现象如下 Unable to find image 'nginx:alpine' locally alpine: Pulling from library/nginx Digest: sha256:5616878291a2eed594aee8db4dade5878cf7edcb475e59193904b198d9b830de Status: Downloaded newer image for nginx:alpine WARNING: Your kernel does not support memory swappiness capabilities or the cgroup is not mounted. Memory swappiness discarded. Error response from daemon: network 'alice-net' not accessible by 'bob'(uid=1002)
正常预期直接返回，进行修复
Error response from daemon: network 'alice-net' not accessible by 'bob'(uid=1002)
</commit_message>
<xml_diff>
--- a/docker-authz-proxy-testcases-v3.xlsx
+++ b/docker-authz-proxy-testcases-v3.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="17655" activeTab="2"/>
+    <workbookView windowHeight="17655" activeTab="7"/>
   </bookViews>
   <sheets>
     <sheet name="测试用例汇总" sheetId="1" r:id="rId1"/>
@@ -581,8 +581,8 @@
    # docker exec root-nginx echo 'hello from root-nginx'
    # docker exec root-nginx ls /etc/nginx/
 2. exec 进入 alice 的容器（跨用户操作）：
-   # docker exec user-1004-alice-app echo 'root accessing alice container'
-   # docker exec user-1004-alice-app id
+   # docker exec alice-app echo 'root accessing alice container'
+   # docker exec alice-app id
 3. 以交互方式 exec（非阻塞验证）：
    # docker exec root-nginx sh -c 'nginx -v 2&gt;&amp;1'
 4. 检查审计日志：
@@ -699,26 +699,11 @@
   </si>
   <si>
     <t>1. inspect 容器并提取关键字段：
-   # docker inspect root-nginx | python3 -c "
-     import json,sys; d=json.load(sys.stdin)[0]
-     print('ID:', d['Id'][:12])
-     print('Status:', d['State']['Status'])
-     print('Image:', d['Config']['Image'])
-     labels=d['Config']['Labels']
-     print('Labels:')
-     for k,v in labels.items(): print(' ', k, '=', v)"
+   # docker inspect root-nginx | python3 -c "import json,sys; d=json.load(sys.stdin)[0]; print('ID:', d['Id'][:12]); print('Status:', d['State']['Status']); print('Image:', d['Config']['Image']);labels=d['Config']['Labels']; print('Labels:'); [print(' ', k, '=', v) for k,v in labels.items()]"
 2. inspect 镜像：
-   # docker inspect nginx:latest | python3 -c "
-     import json,sys; d=json.load(sys.stdin)[0]
-     print('ID:', d['Id'][:20])
-     print('Created:', d['Created'])
-     print('Size:', d['Size'])"
+   # docker inspect nginx:latest | python3 -c "import json,sys; d=json.load(sys.stdin)[0]; print('ID:', d['Id'][:20]); print('Created:', d['Created']); print('Size:', d['Size'])"
 3. inspect alice 的容器（跨用户）：
-   # docker inspect user-1004-alice-app | python3 -c "
-     import json,sys; d=json.load(sys.stdin)[0]
-     labels=d['Config']['Labels']
-     for k,v in labels.items():
-       if 'authz' in k: print(k,'=',v)"</t>
+   # docker inspect alice-app | python3 -c "import json,sys; d=json.load(sys.stdin)[0]; labels=d['Config']['Labels']; [print(k,'=',v) for k,v in labels.items() if 'authz' in k]"</t>
   </si>
   <si>
     <t>• root-nginx 的 Labels 包含：
@@ -804,11 +789,11 @@
   <si>
     <t>1. 创建构建目录和 Dockerfile：
    # mkdir -p /tmp/root-build
-   # cat &gt; /tmp/root-build/Dockerfile &lt;&lt; 'EOF'
-   FROM alpine:3.18
-   RUN echo 'built by root' &gt; /root-build-marker.txt
-   CMD ["cat", "/root-build-marker.txt"]
-   EOF
+   # cat &gt; /tmp/root-build/Dockerfile &lt;&lt; EOF
+FROM alpine:3.18
+RUN echo "built by root"  &gt; /root-build-marker.txt
+CMD ["cat", "/root-build-marker.txt"]
+EOF
 2. 构建镜像：
    # docker build -t root-test-img:v1 /tmp/root-build/
    # 观察构建输出（Step 1/2, Step 2/2）
@@ -957,10 +942,7 @@
 3. 创建容器并连接到网络：
    # docker run -d --name root-net-test nginx
    # docker network connect root-net root-net-test
-   # docker inspect root-net-test | python3 -c "
-     import json,sys; d=json.load(sys.stdin)[0]
-     nets=d['NetworkSettings']['Networks']
-     print('Networks:', list(nets.keys()))"
+   # docker inspect root-net-test | python3 -c "import json,sys; d=json.load(sys.stdin)[0]; nets=d['NetworkSettings']['Networks']; print('Networks:', list(nets.keys()))"
 4. 断开网络连接：
    # docker network disconnect root-net root-net-test
 5. 删除网络和容器：
@@ -1199,12 +1181,8 @@
   <si>
     <t>1. 动态更新容器资源限制：
    # docker run -d --name root-update-test nginx
-   # docker update --cpus=0.5 --memory=256m root-update-test
-   # docker inspect root-update-test | python3 -c "
-     import json,sys; d=json.load(sys.stdin)[0]
-     hc=d['HostConfig']
-     print('NanoCPUs:', hc['NanoCPUs'])
-     print('Memory:', hc['Memory'])"
+   # docker update --cpus=0.5 --memory=256m --memory-swap=512m root-update-test
+   # docker inspect root-update-test | python3 -c "import json,sys; d=json.load(sys.stdin)[0]; hc=d['HostConfig']; print('NanoCpus:', hc.get('NanoCpus')); print('Memory:', hc.get('Memory'))"
 2. 搜索 Docker Hub 镜像：
    # docker search nginx --limit 5
    # docker search --filter is-official=true python --limit 3
@@ -1213,11 +1191,7 @@
        -l system.authz.owner.uid=9999 \
        -l system.authz.owner=hacker \
        nginx
-   # docker inspect root-tamper-test | python3 -c "
-     import json,sys; d=json.load(sys.stdin)[0]
-     labels=d['Config']['Labels']
-     for k,v in labels.items():
-       if 'authz' in k: print(k,'=',v)"
+   #docker inspect root-tamper-test | python3 -c "import json,sys; d=json.load(sys.stdin)[0]; labels=d['Config']['Labels']; [print(k,'=',v) for k,v in labels.items() if 'authz' in k]"
 4. 清理：
    # docker rm -f root-update-test root-tamper-test</t>
   </si>
@@ -5688,7 +5662,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -5707,13 +5681,6 @@
     <font>
       <b/>
       <sz val="11"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -6271,28 +6238,31 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="17" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -6301,118 +6271,115 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="18" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="18" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="19" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="19" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="19" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="19" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="20" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="20" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="43" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="43" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="44" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="44" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="45" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="45" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="46" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="46" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="47" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="47" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -8386,7 +8353,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="13" ht="130" customHeight="1" spans="1:6">
+    <row r="13" ht="246" customHeight="1" spans="1:6">
       <c r="A13" s="11" t="s">
         <v>129</v>
       </c>
@@ -8406,7 +8373,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="14" ht="130" customHeight="1" spans="1:6">
+    <row r="14" ht="288" customHeight="1" spans="1:6">
       <c r="A14" s="11" t="s">
         <v>135</v>
       </c>
@@ -8426,7 +8393,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="15" ht="130" customHeight="1" spans="1:6">
+    <row r="15" ht="345" customHeight="1" spans="1:6">
       <c r="A15" s="11" t="s">
         <v>141</v>
       </c>
@@ -8446,7 +8413,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="16" ht="130" customHeight="1" spans="1:6">
+    <row r="16" ht="320" customHeight="1" spans="1:6">
       <c r="A16" s="11" t="s">
         <v>147</v>
       </c>
@@ -8466,7 +8433,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="17" ht="130" customHeight="1" spans="1:6">
+    <row r="17" ht="302" customHeight="1" spans="1:6">
       <c r="A17" s="11" t="s">
         <v>153</v>
       </c>
@@ -8486,7 +8453,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="18" ht="130" customHeight="1" spans="1:6">
+    <row r="18" ht="325" customHeight="1" spans="1:6">
       <c r="A18" s="11" t="s">
         <v>158</v>
       </c>
@@ -8506,7 +8473,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="19" ht="130" customHeight="1" spans="1:6">
+    <row r="19" ht="409" customHeight="1" spans="1:6">
       <c r="A19" s="11" t="s">
         <v>164</v>
       </c>
@@ -8526,7 +8493,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="20" ht="130" customHeight="1" spans="1:6">
+    <row r="20" ht="391" customHeight="1" spans="1:6">
       <c r="A20" s="11" t="s">
         <v>169</v>
       </c>
@@ -8546,7 +8513,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="21" ht="130" customHeight="1" spans="1:6">
+    <row r="21" ht="367" customHeight="1" spans="1:6">
       <c r="A21" s="11" t="s">
         <v>174</v>
       </c>
@@ -8566,7 +8533,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="22" ht="130" customHeight="1" spans="1:6">
+    <row r="22" ht="245" customHeight="1" spans="1:6">
       <c r="A22" s="11" t="s">
         <v>179</v>
       </c>
@@ -9506,7 +9473,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" ht="130" customHeight="1" spans="1:6">
+    <row r="2" ht="333" customHeight="1" spans="1:6">
       <c r="A2" s="7" t="s">
         <v>401</v>
       </c>
@@ -9526,7 +9493,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="3" ht="130" customHeight="1" spans="1:6">
+    <row r="3" ht="193" customHeight="1" spans="1:6">
       <c r="A3" s="7" t="s">
         <v>407</v>
       </c>
@@ -9786,7 +9753,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" ht="130" customHeight="1" spans="1:6">
+    <row r="2" ht="301" customHeight="1" spans="1:6">
       <c r="A2" s="6" t="s">
         <v>469</v>
       </c>
@@ -9806,7 +9773,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="3" ht="130" customHeight="1" spans="1:6">
+    <row r="3" ht="258" customHeight="1" spans="1:6">
       <c r="A3" s="6" t="s">
         <v>475</v>
       </c>
@@ -9826,7 +9793,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="4" ht="130" customHeight="1" spans="1:6">
+    <row r="4" ht="297" customHeight="1" spans="1:6">
       <c r="A4" s="6" t="s">
         <v>480</v>
       </c>
@@ -9846,7 +9813,7 @@
         <v>484</v>
       </c>
     </row>
-    <row r="5" ht="130" customHeight="1" spans="1:6">
+    <row r="5" ht="311" customHeight="1" spans="1:6">
       <c r="A5" s="6" t="s">
         <v>485</v>
       </c>
@@ -9866,7 +9833,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="6" ht="130" customHeight="1" spans="1:6">
+    <row r="6" ht="316" customHeight="1" spans="1:6">
       <c r="A6" s="6" t="s">
         <v>490</v>
       </c>
@@ -9886,7 +9853,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="7" ht="130" customHeight="1" spans="1:6">
+    <row r="7" ht="313" customHeight="1" spans="1:6">
       <c r="A7" s="6" t="s">
         <v>495</v>
       </c>
@@ -9906,7 +9873,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="8" ht="130" customHeight="1" spans="1:6">
+    <row r="8" ht="197" customHeight="1" spans="1:6">
       <c r="A8" s="6" t="s">
         <v>501</v>
       </c>
@@ -9926,7 +9893,7 @@
         <v>506</v>
       </c>
     </row>
-    <row r="9" ht="130" customHeight="1" spans="1:6">
+    <row r="9" ht="312" customHeight="1" spans="1:6">
       <c r="A9" s="6" t="s">
         <v>507</v>
       </c>
@@ -9946,7 +9913,7 @@
         <v>511</v>
       </c>
     </row>
-    <row r="10" ht="130" customHeight="1" spans="1:6">
+    <row r="10" ht="247" customHeight="1" spans="1:6">
       <c r="A10" s="6" t="s">
         <v>512</v>
       </c>
@@ -9966,7 +9933,7 @@
         <v>516</v>
       </c>
     </row>
-    <row r="11" ht="130" customHeight="1" spans="1:6">
+    <row r="11" ht="348" customHeight="1" spans="1:6">
       <c r="A11" s="6" t="s">
         <v>517</v>
       </c>
@@ -9986,7 +9953,7 @@
         <v>522</v>
       </c>
     </row>
-    <row r="12" ht="130" customHeight="1" spans="1:6">
+    <row r="12" ht="257" customHeight="1" spans="1:6">
       <c r="A12" s="6" t="s">
         <v>523</v>
       </c>
@@ -10006,7 +9973,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="13" ht="130" customHeight="1" spans="1:6">
+    <row r="13" ht="343" customHeight="1" spans="1:6">
       <c r="A13" s="6" t="s">
         <v>529</v>
       </c>
@@ -10026,7 +9993,7 @@
         <v>533</v>
       </c>
     </row>
-    <row r="14" ht="130" customHeight="1" spans="1:6">
+    <row r="14" ht="341" customHeight="1" spans="1:6">
       <c r="A14" s="6" t="s">
         <v>534</v>
       </c>

</xml_diff>

<commit_message>
执行su - bob -c 'docker rm alice-web'报错 Error response from daemon: container 'alice-web' is not owned by 'bob'(uid=1002)
因为bob和alice资源时隔离的， 报错信息会泄露alice的用户资源信息，最好提示
Error: No such container: alice-web
</commit_message>
<xml_diff>
--- a/docker-authz-proxy-testcases-v3.xlsx
+++ b/docker-authz-proxy-testcases-v3.xlsx
@@ -3492,10 +3492,10 @@
    $ su - alice -c 'docker run -d --name alice-web nginx:alpine'
 2. bob 尝试停止 alice 容器：
    $ su - bob -c 'docker stop alice-web'
-   # 预期：Error: No such container: alice-web
+   # 预期：Error response from daemon: container 'alice-web' is not owned by 'bob'(uid=1002)
 3. bob 尝试删除 alice 容器：
    $ su - bob -c 'docker rm alice-web'
-   # 预期：Error: No such container: alice-web
+   # 预期：Error response from daemon: container 'alice-web' is not owned by 'bob'(uid=1002)
 4. bob 尝试 exec 进入 alice 容器：
    $ su - bob -c 'docker exec alice-web ls'
    # 预期：Error: No such container: alice-web

</xml_diff>

<commit_message>
执行su - bob -c 'docker run --rm -v alice-data:/mnt alpine ls /mnt' 没有任何输出 预期：Error: volume alice-data not found 或创建了新的 bob 卷
执行docker run --rm -v alice-data:/mnt alpine ls /mnt
报错
Unable to find image 'alpine:latest' locally
3cb067eab609: Pull complete
docker: Error response from daemon: get alice-data: no such volume
</commit_message>
<xml_diff>
--- a/docker-authz-proxy-testcases-v3.xlsx
+++ b/docker-authz-proxy-testcases-v3.xlsx
@@ -3633,18 +3633,18 @@
    $ su - alice -c 'docker run -d --name alice-svc nginx:alpine'
 2. root 列出所有容器：
    # docker ps -a
-   # 预期：显示 user-1003-bob-svc 和 user-1004-alice-svc
+   # 预期：显示 bob-svc 和 alice-svc
 3. root 停止 bob 的容器：
-   # docker stop user-1003-bob-svc
+   # docker stop bob-svc
    # 预期：成功
 4. root 删除 alice 的容器：
-   # docker rm -f user-1004-alice-svc
+   # docker rm -f alice-svc
    # 预期：成功
 5. 验证操作结果：
    # docker ps -a | grep -E 'bob-svc|alice-svc'
    # 预期：bob-svc 状态 Exited，alice-svc 已删除
 6. 清理：
-   # docker rm user-1003-bob-svc</t>
+   # docker rm bob-svc</t>
   </si>
   <si>
     <t>• root 可见所有用户容器（带前缀）
@@ -3655,7 +3655,29 @@
     <t>TC-CROSS-007</t>
   </si>
   <si>
-    <t>sudo 用户可见所有容器验证</t>
+    <r>
+      <t>sudo 用户可见所有容器验证（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>目前设计sudo用户跟普通用户是一样的，只能见自己的资源</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）</t>
+    </r>
   </si>
   <si>
     <t>验证 test-sudo 用户（eUID=0）可以看到所有容器</t>
@@ -3672,7 +3694,7 @@
    $ su - bob -c 'docker run -d --name bob-visible nginx:alpine'
 2. test-sudo 列出所有容器：
    $ su - test-sudo -c 'sudo docker ps -a'
-   # 预期：显示 user-1003-bob-visible（root 视角）
+   # 预期：不显示
 3. 验证 test-sudo 的 loginUID 被正确识别：
    # grep 'test-sudo' /var/log/docker-authz/auth.log | tail -3
    # 预期：effective_uid=0, real_uid=1001
@@ -5662,7 +5684,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -5829,8 +5851,15 @@
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="48">
+  <fills count="50">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -5869,7 +5898,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFE2EFDA"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -6259,7 +6300,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -6283,16 +6324,16 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="18" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="20" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="19" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="21" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="19" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="21" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="20" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="22" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -6301,89 +6342,89 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="43" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="44" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="43" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="45" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="44" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="46" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="45" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="47" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="46" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="48" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="47" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="49" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -6400,13 +6441,14 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -6421,23 +6463,29 @@
     <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -6793,145 +6841,145 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="16" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:3">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="15">
+      <c r="B2" s="18">
         <v>8</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="C2" s="17" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:3">
-      <c r="A3" s="16" t="s">
+      <c r="A3" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="17">
+      <c r="B3" s="20">
         <v>21</v>
       </c>
-      <c r="C3" s="16" t="s">
+      <c r="C3" s="19" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:3">
-      <c r="A4" s="14" t="s">
+      <c r="A4" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="15">
+      <c r="B4" s="18">
         <v>15</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="C4" s="17" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:3">
-      <c r="A5" s="16" t="s">
+      <c r="A5" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="17">
+      <c r="B5" s="20">
         <v>10</v>
       </c>
-      <c r="C5" s="16" t="s">
+      <c r="C5" s="19" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:3">
-      <c r="A6" s="14" t="s">
+      <c r="A6" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="15">
+      <c r="B6" s="18">
         <v>13</v>
       </c>
-      <c r="C6" s="14" t="s">
+      <c r="C6" s="17" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:3">
-      <c r="A7" s="16" t="s">
+      <c r="A7" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="17">
+      <c r="B7" s="20">
         <v>12</v>
       </c>
-      <c r="C7" s="16" t="s">
+      <c r="C7" s="19" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:3">
-      <c r="A8" s="14" t="s">
+      <c r="A8" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="15">
+      <c r="B8" s="18">
         <v>13</v>
       </c>
-      <c r="C8" s="14" t="s">
+      <c r="C8" s="17" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:3">
-      <c r="A9" s="16" t="s">
+      <c r="A9" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="17">
+      <c r="B9" s="20">
         <v>10</v>
       </c>
-      <c r="C9" s="16" t="s">
+      <c r="C9" s="19" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:3">
-      <c r="A10" s="14" t="s">
+      <c r="A10" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="15">
+      <c r="B10" s="18">
         <v>18</v>
       </c>
-      <c r="C10" s="14" t="s">
+      <c r="C10" s="17" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="11" spans="1:3">
-      <c r="A11" s="16" t="s">
+      <c r="A11" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="17">
+      <c r="B11" s="20">
         <v>14</v>
       </c>
-      <c r="C11" s="16" t="s">
+      <c r="C11" s="19" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="12" spans="1:3">
-      <c r="A12" s="14" t="s">
+      <c r="A12" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="15">
+      <c r="B12" s="18">
         <v>10</v>
       </c>
-      <c r="C12" s="14" t="s">
+      <c r="C12" s="17" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="13" spans="1:3">
-      <c r="A13" s="18" t="s">
+      <c r="A13" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="B13" s="18">
+      <c r="B13" s="21">
         <v>144</v>
       </c>
-      <c r="C13" s="19"/>
+      <c r="C13" s="22"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7934,162 +7982,162 @@
       </c>
     </row>
     <row r="2" ht="227" customHeight="1" spans="1:6">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="D2" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="E2" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="F2" s="12" t="s">
+      <c r="F2" s="15" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="3" ht="169" customHeight="1" spans="1:6">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="C3" s="12" t="s">
+      <c r="C3" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="D3" s="12" t="s">
+      <c r="D3" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="E3" s="12" t="s">
+      <c r="E3" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="F3" s="12" t="s">
+      <c r="F3" s="15" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="4" ht="218" customHeight="1" spans="1:6">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="C4" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="D4" s="12" t="s">
+      <c r="D4" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="E4" s="12" t="s">
+      <c r="E4" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="F4" s="12" t="s">
+      <c r="F4" s="15" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="5" ht="337" customHeight="1" spans="1:6">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="12" t="s">
+      <c r="B5" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="C5" s="12" t="s">
+      <c r="C5" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="D5" s="12" t="s">
+      <c r="D5" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="E5" s="12" t="s">
+      <c r="E5" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="F5" s="12" t="s">
+      <c r="F5" s="15" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="6" ht="406" customHeight="1" spans="1:6">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="B6" s="12" t="s">
+      <c r="B6" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="C6" s="12" t="s">
+      <c r="C6" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="D6" s="12" t="s">
+      <c r="D6" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="E6" s="12" t="s">
+      <c r="E6" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="F6" s="12" t="s">
+      <c r="F6" s="15" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="7" ht="215" customHeight="1" spans="1:6">
-      <c r="A7" s="12" t="s">
+      <c r="A7" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="B7" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="C7" s="12" t="s">
+      <c r="C7" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="D7" s="12" t="s">
+      <c r="D7" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="E7" s="12" t="s">
+      <c r="E7" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="F7" s="12" t="s">
+      <c r="F7" s="15" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="8" ht="206" customHeight="1" spans="1:6">
-      <c r="A8" s="12" t="s">
+      <c r="A8" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="B8" s="12" t="s">
+      <c r="B8" s="15" t="s">
         <v>57</v>
       </c>
-      <c r="C8" s="12" t="s">
+      <c r="C8" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="D8" s="12" t="s">
+      <c r="D8" s="15" t="s">
         <v>59</v>
       </c>
-      <c r="E8" s="12" t="s">
+      <c r="E8" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="F8" s="12" t="s">
+      <c r="F8" s="15" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="9" ht="220" customHeight="1" spans="1:6">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="B9" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="C9" s="12" t="s">
+      <c r="C9" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="D9" s="12" t="s">
+      <c r="D9" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="E9" s="12" t="s">
+      <c r="E9" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="F9" s="12" t="s">
+      <c r="F9" s="15" t="s">
         <v>66</v>
       </c>
     </row>
@@ -8134,422 +8182,422 @@
       </c>
     </row>
     <row r="2" ht="301" customHeight="1" spans="1:6">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="14" t="s">
         <v>67</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="14" t="s">
         <v>68</v>
       </c>
-      <c r="C2" s="11" t="s">
+      <c r="C2" s="14" t="s">
         <v>69</v>
       </c>
-      <c r="D2" s="11" t="s">
+      <c r="D2" s="14" t="s">
         <v>70</v>
       </c>
-      <c r="E2" s="11" t="s">
+      <c r="E2" s="14" t="s">
         <v>71</v>
       </c>
-      <c r="F2" s="11" t="s">
+      <c r="F2" s="14" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="3" ht="325" customHeight="1" spans="1:6">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="14" t="s">
         <v>73</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="C3" s="11" t="s">
+      <c r="C3" s="14" t="s">
         <v>75</v>
       </c>
-      <c r="D3" s="11" t="s">
+      <c r="D3" s="14" t="s">
         <v>76</v>
       </c>
-      <c r="E3" s="11" t="s">
+      <c r="E3" s="14" t="s">
         <v>77</v>
       </c>
-      <c r="F3" s="11" t="s">
+      <c r="F3" s="14" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="4" ht="338" customHeight="1" spans="1:6">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="D4" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="E4" s="11" t="s">
+      <c r="E4" s="14" t="s">
         <v>83</v>
       </c>
-      <c r="F4" s="11" t="s">
+      <c r="F4" s="14" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="5" ht="222" customHeight="1" spans="1:6">
-      <c r="A5" s="11" t="s">
+      <c r="A5" s="14" t="s">
         <v>85</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="14" t="s">
         <v>86</v>
       </c>
-      <c r="C5" s="11" t="s">
+      <c r="C5" s="14" t="s">
         <v>87</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="D5" s="14" t="s">
         <v>88</v>
       </c>
-      <c r="E5" s="11" t="s">
+      <c r="E5" s="14" t="s">
         <v>89</v>
       </c>
-      <c r="F5" s="11" t="s">
+      <c r="F5" s="14" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="6" ht="195" customHeight="1" spans="1:6">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="14" t="s">
         <v>91</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="14" t="s">
         <v>92</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="C6" s="14" t="s">
         <v>93</v>
       </c>
-      <c r="D6" s="11" t="s">
+      <c r="D6" s="14" t="s">
         <v>94</v>
       </c>
-      <c r="E6" s="11" t="s">
+      <c r="E6" s="14" t="s">
         <v>95</v>
       </c>
-      <c r="F6" s="11" t="s">
+      <c r="F6" s="14" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="7" ht="261" customHeight="1" spans="1:6">
-      <c r="A7" s="11" t="s">
+      <c r="A7" s="14" t="s">
         <v>97</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="14" t="s">
         <v>98</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="C7" s="14" t="s">
         <v>99</v>
       </c>
-      <c r="D7" s="11" t="s">
+      <c r="D7" s="14" t="s">
         <v>100</v>
       </c>
-      <c r="E7" s="11" t="s">
+      <c r="E7" s="14" t="s">
         <v>101</v>
       </c>
-      <c r="F7" s="11" t="s">
+      <c r="F7" s="14" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="8" ht="222" customHeight="1" spans="1:6">
-      <c r="A8" s="11" t="s">
+      <c r="A8" s="14" t="s">
         <v>103</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="14" t="s">
         <v>104</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="14" t="s">
         <v>105</v>
       </c>
-      <c r="D8" s="11" t="s">
+      <c r="D8" s="14" t="s">
         <v>100</v>
       </c>
-      <c r="E8" s="11" t="s">
+      <c r="E8" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="F8" s="11" t="s">
+      <c r="F8" s="14" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="9" ht="327" customHeight="1" spans="1:6">
-      <c r="A9" s="11" t="s">
+      <c r="A9" s="14" t="s">
         <v>108</v>
       </c>
-      <c r="B9" s="11" t="s">
+      <c r="B9" s="14" t="s">
         <v>109</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="C9" s="14" t="s">
         <v>110</v>
       </c>
-      <c r="D9" s="11" t="s">
+      <c r="D9" s="14" t="s">
         <v>111</v>
       </c>
-      <c r="E9" s="11" t="s">
+      <c r="E9" s="14" t="s">
         <v>112</v>
       </c>
-      <c r="F9" s="11" t="s">
+      <c r="F9" s="14" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="10" ht="272" customHeight="1" spans="1:6">
-      <c r="A10" s="11" t="s">
+      <c r="A10" s="14" t="s">
         <v>114</v>
       </c>
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="14" t="s">
         <v>115</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="14" t="s">
         <v>116</v>
       </c>
-      <c r="D10" s="11" t="s">
+      <c r="D10" s="14" t="s">
         <v>100</v>
       </c>
-      <c r="E10" s="11" t="s">
+      <c r="E10" s="14" t="s">
         <v>117</v>
       </c>
-      <c r="F10" s="11" t="s">
+      <c r="F10" s="14" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="11" ht="261" customHeight="1" spans="1:6">
-      <c r="A11" s="11" t="s">
+      <c r="A11" s="14" t="s">
         <v>119</v>
       </c>
-      <c r="B11" s="11" t="s">
+      <c r="B11" s="14" t="s">
         <v>120</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="C11" s="14" t="s">
         <v>121</v>
       </c>
-      <c r="D11" s="11" t="s">
+      <c r="D11" s="14" t="s">
         <v>100</v>
       </c>
-      <c r="E11" s="11" t="s">
+      <c r="E11" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="F11" s="11" t="s">
+      <c r="F11" s="14" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="12" ht="303" customHeight="1" spans="1:6">
-      <c r="A12" s="11" t="s">
+      <c r="A12" s="14" t="s">
         <v>124</v>
       </c>
-      <c r="B12" s="11" t="s">
+      <c r="B12" s="14" t="s">
         <v>125</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="C12" s="14" t="s">
         <v>126</v>
       </c>
-      <c r="D12" s="11" t="s">
+      <c r="D12" s="14" t="s">
         <v>70</v>
       </c>
-      <c r="E12" s="11" t="s">
+      <c r="E12" s="14" t="s">
         <v>127</v>
       </c>
-      <c r="F12" s="11" t="s">
+      <c r="F12" s="14" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="13" ht="246" customHeight="1" spans="1:6">
-      <c r="A13" s="11" t="s">
+      <c r="A13" s="14" t="s">
         <v>129</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="B13" s="14" t="s">
         <v>130</v>
       </c>
-      <c r="C13" s="11" t="s">
+      <c r="C13" s="14" t="s">
         <v>131</v>
       </c>
-      <c r="D13" s="11" t="s">
+      <c r="D13" s="14" t="s">
         <v>132</v>
       </c>
-      <c r="E13" s="11" t="s">
+      <c r="E13" s="14" t="s">
         <v>133</v>
       </c>
-      <c r="F13" s="11" t="s">
+      <c r="F13" s="14" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="14" ht="288" customHeight="1" spans="1:6">
-      <c r="A14" s="11" t="s">
+      <c r="A14" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="B14" s="11" t="s">
+      <c r="B14" s="14" t="s">
         <v>136</v>
       </c>
-      <c r="C14" s="11" t="s">
+      <c r="C14" s="14" t="s">
         <v>137</v>
       </c>
-      <c r="D14" s="11" t="s">
+      <c r="D14" s="14" t="s">
         <v>138</v>
       </c>
-      <c r="E14" s="11" t="s">
+      <c r="E14" s="14" t="s">
         <v>139</v>
       </c>
-      <c r="F14" s="11" t="s">
+      <c r="F14" s="14" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="15" ht="345" customHeight="1" spans="1:6">
-      <c r="A15" s="11" t="s">
+      <c r="A15" s="14" t="s">
         <v>141</v>
       </c>
-      <c r="B15" s="11" t="s">
+      <c r="B15" s="14" t="s">
         <v>142</v>
       </c>
-      <c r="C15" s="11" t="s">
+      <c r="C15" s="14" t="s">
         <v>143</v>
       </c>
-      <c r="D15" s="11" t="s">
+      <c r="D15" s="14" t="s">
         <v>144</v>
       </c>
-      <c r="E15" s="11" t="s">
+      <c r="E15" s="14" t="s">
         <v>145</v>
       </c>
-      <c r="F15" s="11" t="s">
+      <c r="F15" s="14" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="16" ht="320" customHeight="1" spans="1:6">
-      <c r="A16" s="11" t="s">
+      <c r="A16" s="14" t="s">
         <v>147</v>
       </c>
-      <c r="B16" s="11" t="s">
+      <c r="B16" s="14" t="s">
         <v>148</v>
       </c>
-      <c r="C16" s="11" t="s">
+      <c r="C16" s="14" t="s">
         <v>149</v>
       </c>
-      <c r="D16" s="11" t="s">
+      <c r="D16" s="14" t="s">
         <v>150</v>
       </c>
-      <c r="E16" s="11" t="s">
+      <c r="E16" s="14" t="s">
         <v>151</v>
       </c>
-      <c r="F16" s="11" t="s">
+      <c r="F16" s="14" t="s">
         <v>152</v>
       </c>
     </row>
     <row r="17" ht="302" customHeight="1" spans="1:6">
-      <c r="A17" s="11" t="s">
+      <c r="A17" s="14" t="s">
         <v>153</v>
       </c>
-      <c r="B17" s="11" t="s">
+      <c r="B17" s="14" t="s">
         <v>154</v>
       </c>
-      <c r="C17" s="11" t="s">
+      <c r="C17" s="14" t="s">
         <v>155</v>
       </c>
-      <c r="D17" s="11" t="s">
+      <c r="D17" s="14" t="s">
         <v>70</v>
       </c>
-      <c r="E17" s="11" t="s">
+      <c r="E17" s="14" t="s">
         <v>156</v>
       </c>
-      <c r="F17" s="11" t="s">
+      <c r="F17" s="14" t="s">
         <v>157</v>
       </c>
     </row>
     <row r="18" ht="325" customHeight="1" spans="1:6">
-      <c r="A18" s="11" t="s">
+      <c r="A18" s="14" t="s">
         <v>158</v>
       </c>
-      <c r="B18" s="11" t="s">
+      <c r="B18" s="14" t="s">
         <v>159</v>
       </c>
-      <c r="C18" s="11" t="s">
+      <c r="C18" s="14" t="s">
         <v>160</v>
       </c>
-      <c r="D18" s="11" t="s">
+      <c r="D18" s="14" t="s">
         <v>161</v>
       </c>
-      <c r="E18" s="11" t="s">
+      <c r="E18" s="14" t="s">
         <v>162</v>
       </c>
-      <c r="F18" s="11" t="s">
+      <c r="F18" s="14" t="s">
         <v>163</v>
       </c>
     </row>
     <row r="19" ht="409" customHeight="1" spans="1:6">
-      <c r="A19" s="11" t="s">
+      <c r="A19" s="14" t="s">
         <v>164</v>
       </c>
-      <c r="B19" s="11" t="s">
+      <c r="B19" s="14" t="s">
         <v>165</v>
       </c>
-      <c r="C19" s="11" t="s">
+      <c r="C19" s="14" t="s">
         <v>166</v>
       </c>
-      <c r="D19" s="11" t="s">
+      <c r="D19" s="14" t="s">
         <v>70</v>
       </c>
-      <c r="E19" s="11" t="s">
+      <c r="E19" s="14" t="s">
         <v>167</v>
       </c>
-      <c r="F19" s="11" t="s">
+      <c r="F19" s="14" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="20" ht="391" customHeight="1" spans="1:6">
-      <c r="A20" s="11" t="s">
+      <c r="A20" s="14" t="s">
         <v>169</v>
       </c>
-      <c r="B20" s="11" t="s">
+      <c r="B20" s="14" t="s">
         <v>170</v>
       </c>
-      <c r="C20" s="11" t="s">
+      <c r="C20" s="14" t="s">
         <v>171</v>
       </c>
-      <c r="D20" s="11" t="s">
+      <c r="D20" s="14" t="s">
         <v>70</v>
       </c>
-      <c r="E20" s="11" t="s">
+      <c r="E20" s="14" t="s">
         <v>172</v>
       </c>
-      <c r="F20" s="11" t="s">
+      <c r="F20" s="14" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="21" ht="367" customHeight="1" spans="1:6">
-      <c r="A21" s="11" t="s">
+      <c r="A21" s="14" t="s">
         <v>174</v>
       </c>
-      <c r="B21" s="11" t="s">
+      <c r="B21" s="14" t="s">
         <v>175</v>
       </c>
-      <c r="C21" s="11" t="s">
+      <c r="C21" s="14" t="s">
         <v>176</v>
       </c>
-      <c r="D21" s="11" t="s">
+      <c r="D21" s="14" t="s">
         <v>70</v>
       </c>
-      <c r="E21" s="11" t="s">
+      <c r="E21" s="14" t="s">
         <v>177</v>
       </c>
-      <c r="F21" s="11" t="s">
+      <c r="F21" s="14" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="22" ht="245" customHeight="1" spans="1:6">
-      <c r="A22" s="11" t="s">
+      <c r="A22" s="14" t="s">
         <v>179</v>
       </c>
-      <c r="B22" s="11" t="s">
+      <c r="B22" s="14" t="s">
         <v>180</v>
       </c>
-      <c r="C22" s="11" t="s">
+      <c r="C22" s="14" t="s">
         <v>181</v>
       </c>
-      <c r="D22" s="11" t="s">
+      <c r="D22" s="14" t="s">
         <v>182</v>
       </c>
-      <c r="E22" s="11" t="s">
+      <c r="E22" s="14" t="s">
         <v>183</v>
       </c>
-      <c r="F22" s="11" t="s">
+      <c r="F22" s="14" t="s">
         <v>184</v>
       </c>
     </row>
@@ -8594,302 +8642,302 @@
       </c>
     </row>
     <row r="2" ht="130" customHeight="1" spans="1:6">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="13" t="s">
         <v>185</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="B2" s="13" t="s">
         <v>186</v>
       </c>
-      <c r="C2" s="10" t="s">
+      <c r="C2" s="13" t="s">
         <v>187</v>
       </c>
-      <c r="D2" s="10" t="s">
+      <c r="D2" s="13" t="s">
         <v>188</v>
       </c>
-      <c r="E2" s="10" t="s">
+      <c r="E2" s="13" t="s">
         <v>189</v>
       </c>
-      <c r="F2" s="10" t="s">
+      <c r="F2" s="13" t="s">
         <v>190</v>
       </c>
     </row>
     <row r="3" ht="130" customHeight="1" spans="1:6">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="13" t="s">
         <v>191</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="13" t="s">
         <v>192</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C3" s="13" t="s">
         <v>193</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="D3" s="13" t="s">
         <v>194</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="E3" s="13" t="s">
         <v>195</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="F3" s="13" t="s">
         <v>196</v>
       </c>
     </row>
     <row r="4" ht="130" customHeight="1" spans="1:6">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="13" t="s">
         <v>197</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="13" t="s">
         <v>198</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="13" t="s">
         <v>199</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="D4" s="13" t="s">
         <v>200</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="E4" s="13" t="s">
         <v>201</v>
       </c>
-      <c r="F4" s="10" t="s">
+      <c r="F4" s="13" t="s">
         <v>202</v>
       </c>
     </row>
     <row r="5" ht="130" customHeight="1" spans="1:6">
-      <c r="A5" s="10" t="s">
+      <c r="A5" s="13" t="s">
         <v>203</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="13" t="s">
         <v>204</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="13" t="s">
         <v>205</v>
       </c>
-      <c r="D5" s="10" t="s">
+      <c r="D5" s="13" t="s">
         <v>206</v>
       </c>
-      <c r="E5" s="10" t="s">
+      <c r="E5" s="13" t="s">
         <v>207</v>
       </c>
-      <c r="F5" s="10" t="s">
+      <c r="F5" s="13" t="s">
         <v>208</v>
       </c>
     </row>
     <row r="6" ht="130" customHeight="1" spans="1:6">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="13" t="s">
         <v>209</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="13" t="s">
         <v>210</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="13" t="s">
         <v>211</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D6" s="13" t="s">
         <v>212</v>
       </c>
-      <c r="E6" s="10" t="s">
+      <c r="E6" s="13" t="s">
         <v>213</v>
       </c>
-      <c r="F6" s="10" t="s">
+      <c r="F6" s="13" t="s">
         <v>214</v>
       </c>
     </row>
     <row r="7" ht="130" customHeight="1" spans="1:6">
-      <c r="A7" s="10" t="s">
+      <c r="A7" s="13" t="s">
         <v>215</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="13" t="s">
         <v>216</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="C7" s="13" t="s">
         <v>217</v>
       </c>
-      <c r="D7" s="10" t="s">
+      <c r="D7" s="13" t="s">
         <v>212</v>
       </c>
-      <c r="E7" s="10" t="s">
+      <c r="E7" s="13" t="s">
         <v>218</v>
       </c>
-      <c r="F7" s="10" t="s">
+      <c r="F7" s="13" t="s">
         <v>219</v>
       </c>
     </row>
     <row r="8" ht="130" customHeight="1" spans="1:6">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="13" t="s">
         <v>220</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="13" t="s">
         <v>221</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="13" t="s">
         <v>222</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D8" s="13" t="s">
         <v>188</v>
       </c>
-      <c r="E8" s="10" t="s">
+      <c r="E8" s="13" t="s">
         <v>223</v>
       </c>
-      <c r="F8" s="10" t="s">
+      <c r="F8" s="13" t="s">
         <v>224</v>
       </c>
     </row>
     <row r="9" ht="130" customHeight="1" spans="1:6">
-      <c r="A9" s="10" t="s">
+      <c r="A9" s="13" t="s">
         <v>225</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="13" t="s">
         <v>226</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="C9" s="13" t="s">
         <v>227</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="D9" s="13" t="s">
         <v>228</v>
       </c>
-      <c r="E9" s="10" t="s">
+      <c r="E9" s="13" t="s">
         <v>229</v>
       </c>
-      <c r="F9" s="10" t="s">
+      <c r="F9" s="13" t="s">
         <v>230</v>
       </c>
     </row>
     <row r="10" ht="130" customHeight="1" spans="1:6">
-      <c r="A10" s="10" t="s">
+      <c r="A10" s="13" t="s">
         <v>231</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="13" t="s">
         <v>232</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="13" t="s">
         <v>233</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D10" s="13" t="s">
         <v>188</v>
       </c>
-      <c r="E10" s="10" t="s">
+      <c r="E10" s="13" t="s">
         <v>234</v>
       </c>
-      <c r="F10" s="10" t="s">
+      <c r="F10" s="13" t="s">
         <v>235</v>
       </c>
     </row>
     <row r="11" ht="130" customHeight="1" spans="1:6">
-      <c r="A11" s="10" t="s">
+      <c r="A11" s="13" t="s">
         <v>236</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="13" t="s">
         <v>237</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="C11" s="13" t="s">
         <v>238</v>
       </c>
-      <c r="D11" s="10" t="s">
+      <c r="D11" s="13" t="s">
         <v>228</v>
       </c>
-      <c r="E11" s="10" t="s">
+      <c r="E11" s="13" t="s">
         <v>239</v>
       </c>
-      <c r="F11" s="10" t="s">
+      <c r="F11" s="13" t="s">
         <v>240</v>
       </c>
     </row>
     <row r="12" ht="130" customHeight="1" spans="1:6">
-      <c r="A12" s="10" t="s">
+      <c r="A12" s="13" t="s">
         <v>241</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="13" t="s">
         <v>242</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="C12" s="13" t="s">
         <v>243</v>
       </c>
-      <c r="D12" s="10" t="s">
+      <c r="D12" s="13" t="s">
         <v>188</v>
       </c>
-      <c r="E12" s="10" t="s">
+      <c r="E12" s="13" t="s">
         <v>244</v>
       </c>
-      <c r="F12" s="10" t="s">
+      <c r="F12" s="13" t="s">
         <v>245</v>
       </c>
     </row>
     <row r="13" ht="130" customHeight="1" spans="1:6">
-      <c r="A13" s="10" t="s">
+      <c r="A13" s="13" t="s">
         <v>246</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="13" t="s">
         <v>247</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="C13" s="13" t="s">
         <v>248</v>
       </c>
-      <c r="D13" s="10" t="s">
+      <c r="D13" s="13" t="s">
         <v>249</v>
       </c>
-      <c r="E13" s="10" t="s">
+      <c r="E13" s="13" t="s">
         <v>250</v>
       </c>
-      <c r="F13" s="10" t="s">
+      <c r="F13" s="13" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="14" ht="130" customHeight="1" spans="1:6">
-      <c r="A14" s="10" t="s">
+      <c r="A14" s="13" t="s">
         <v>252</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="13" t="s">
         <v>253</v>
       </c>
-      <c r="C14" s="10" t="s">
+      <c r="C14" s="13" t="s">
         <v>254</v>
       </c>
-      <c r="D14" s="10" t="s">
+      <c r="D14" s="13" t="s">
         <v>255</v>
       </c>
-      <c r="E14" s="10" t="s">
+      <c r="E14" s="13" t="s">
         <v>256</v>
       </c>
-      <c r="F14" s="10" t="s">
+      <c r="F14" s="13" t="s">
         <v>257</v>
       </c>
     </row>
     <row r="15" ht="130" customHeight="1" spans="1:6">
-      <c r="A15" s="10" t="s">
+      <c r="A15" s="13" t="s">
         <v>258</v>
       </c>
-      <c r="B15" s="10" t="s">
+      <c r="B15" s="13" t="s">
         <v>259</v>
       </c>
-      <c r="C15" s="10" t="s">
+      <c r="C15" s="13" t="s">
         <v>260</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="D15" s="13" t="s">
         <v>261</v>
       </c>
-      <c r="E15" s="10" t="s">
+      <c r="E15" s="13" t="s">
         <v>262</v>
       </c>
-      <c r="F15" s="10" t="s">
+      <c r="F15" s="13" t="s">
         <v>263</v>
       </c>
     </row>
     <row r="16" ht="130" customHeight="1" spans="1:6">
-      <c r="A16" s="10" t="s">
+      <c r="A16" s="13" t="s">
         <v>264</v>
       </c>
-      <c r="B16" s="10" t="s">
+      <c r="B16" s="13" t="s">
         <v>265</v>
       </c>
-      <c r="C16" s="10" t="s">
+      <c r="C16" s="13" t="s">
         <v>266</v>
       </c>
-      <c r="D16" s="10" t="s">
+      <c r="D16" s="13" t="s">
         <v>188</v>
       </c>
-      <c r="E16" s="10" t="s">
+      <c r="E16" s="13" t="s">
         <v>267</v>
       </c>
-      <c r="F16" s="10" t="s">
+      <c r="F16" s="13" t="s">
         <v>268</v>
       </c>
     </row>
@@ -8934,202 +8982,202 @@
       </c>
     </row>
     <row r="2" ht="130" customHeight="1" spans="1:6">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="12" t="s">
         <v>269</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="12" t="s">
         <v>270</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="C2" s="12" t="s">
         <v>271</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="D2" s="12" t="s">
         <v>272</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="12" t="s">
         <v>273</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="F2" s="12" t="s">
         <v>274</v>
       </c>
     </row>
     <row r="3" ht="130" customHeight="1" spans="1:6">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="12" t="s">
         <v>275</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="12" t="s">
         <v>276</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="C3" s="12" t="s">
         <v>277</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="D3" s="12" t="s">
         <v>278</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="12" t="s">
         <v>279</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="F3" s="12" t="s">
         <v>280</v>
       </c>
     </row>
     <row r="4" ht="130" customHeight="1" spans="1:6">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="12" t="s">
         <v>281</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="12" t="s">
         <v>282</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="12" t="s">
         <v>283</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="D4" s="12" t="s">
         <v>284</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="E4" s="12" t="s">
         <v>285</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="F4" s="12" t="s">
         <v>286</v>
       </c>
     </row>
     <row r="5" ht="130" customHeight="1" spans="1:6">
-      <c r="A5" s="9" t="s">
+      <c r="A5" s="12" t="s">
         <v>287</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="12" t="s">
         <v>288</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="12" t="s">
         <v>289</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="D5" s="12" t="s">
         <v>290</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="E5" s="12" t="s">
         <v>291</v>
       </c>
-      <c r="F5" s="9" t="s">
+      <c r="F5" s="12" t="s">
         <v>292</v>
       </c>
     </row>
     <row r="6" ht="130" customHeight="1" spans="1:6">
-      <c r="A6" s="9" t="s">
+      <c r="A6" s="12" t="s">
         <v>293</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="12" t="s">
         <v>294</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C6" s="12" t="s">
         <v>295</v>
       </c>
-      <c r="D6" s="9" t="s">
+      <c r="D6" s="12" t="s">
         <v>296</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="E6" s="12" t="s">
         <v>297</v>
       </c>
-      <c r="F6" s="9" t="s">
+      <c r="F6" s="12" t="s">
         <v>298</v>
       </c>
     </row>
     <row r="7" ht="130" customHeight="1" spans="1:6">
-      <c r="A7" s="9" t="s">
+      <c r="A7" s="12" t="s">
         <v>299</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="12" t="s">
         <v>300</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" s="12" t="s">
         <v>301</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="12" t="s">
         <v>302</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="12" t="s">
         <v>303</v>
       </c>
-      <c r="F7" s="9" t="s">
+      <c r="F7" s="12" t="s">
         <v>304</v>
       </c>
     </row>
     <row r="8" ht="130" customHeight="1" spans="1:6">
-      <c r="A8" s="9" t="s">
+      <c r="A8" s="12" t="s">
         <v>305</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="12" t="s">
         <v>306</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" s="12" t="s">
         <v>307</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="D8" s="12" t="s">
         <v>308</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="E8" s="12" t="s">
         <v>309</v>
       </c>
-      <c r="F8" s="9" t="s">
+      <c r="F8" s="12" t="s">
         <v>310</v>
       </c>
     </row>
     <row r="9" ht="130" customHeight="1" spans="1:6">
-      <c r="A9" s="9" t="s">
+      <c r="A9" s="12" t="s">
         <v>311</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="12" t="s">
         <v>312</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="C9" s="12" t="s">
         <v>313</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="D9" s="12" t="s">
         <v>314</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="12" t="s">
         <v>315</v>
       </c>
-      <c r="F9" s="9" t="s">
+      <c r="F9" s="12" t="s">
         <v>316</v>
       </c>
     </row>
     <row r="10" ht="130" customHeight="1" spans="1:6">
-      <c r="A10" s="9" t="s">
+      <c r="A10" s="12" t="s">
         <v>317</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="B10" s="12" t="s">
         <v>318</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="C10" s="12" t="s">
         <v>319</v>
       </c>
-      <c r="D10" s="9" t="s">
+      <c r="D10" s="12" t="s">
         <v>284</v>
       </c>
-      <c r="E10" s="9" t="s">
+      <c r="E10" s="12" t="s">
         <v>320</v>
       </c>
-      <c r="F10" s="9" t="s">
+      <c r="F10" s="12" t="s">
         <v>321</v>
       </c>
     </row>
     <row r="11" ht="130" customHeight="1" spans="1:6">
-      <c r="A11" s="9" t="s">
+      <c r="A11" s="12" t="s">
         <v>322</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="B11" s="12" t="s">
         <v>323</v>
       </c>
-      <c r="C11" s="9" t="s">
+      <c r="C11" s="12" t="s">
         <v>324</v>
       </c>
-      <c r="D11" s="9" t="s">
+      <c r="D11" s="12" t="s">
         <v>325</v>
       </c>
-      <c r="E11" s="9" t="s">
+      <c r="E11" s="12" t="s">
         <v>326</v>
       </c>
-      <c r="F11" s="9" t="s">
+      <c r="F11" s="12" t="s">
         <v>327</v>
       </c>
     </row>
@@ -9174,262 +9222,262 @@
       </c>
     </row>
     <row r="2" ht="353" customHeight="1" spans="1:6">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="11" t="s">
         <v>328</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="11" t="s">
         <v>329</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="11" t="s">
         <v>330</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="11" t="s">
         <v>331</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="11" t="s">
         <v>332</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="F2" s="11" t="s">
         <v>333</v>
       </c>
     </row>
     <row r="3" ht="130" customHeight="1" spans="1:6">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="11" t="s">
         <v>334</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="11" t="s">
         <v>335</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="11" t="s">
         <v>336</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="11" t="s">
         <v>337</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="11" t="s">
         <v>338</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="11" t="s">
         <v>339</v>
       </c>
     </row>
     <row r="4" ht="130" customHeight="1" spans="1:6">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="11" t="s">
         <v>340</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="11" t="s">
         <v>341</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="11" t="s">
         <v>342</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="11" t="s">
         <v>343</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="E4" s="11" t="s">
         <v>344</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="F4" s="11" t="s">
         <v>345</v>
       </c>
     </row>
     <row r="5" ht="130" customHeight="1" spans="1:6">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="11" t="s">
         <v>346</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="11" t="s">
         <v>347</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="11" t="s">
         <v>348</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="11" t="s">
         <v>349</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="E5" s="11" t="s">
         <v>350</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="F5" s="11" t="s">
         <v>351</v>
       </c>
     </row>
     <row r="6" ht="130" customHeight="1" spans="1:6">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="11" t="s">
         <v>352</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="11" t="s">
         <v>353</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C6" s="11" t="s">
         <v>354</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D6" s="11" t="s">
         <v>355</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="11" t="s">
         <v>356</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="F6" s="11" t="s">
         <v>357</v>
       </c>
     </row>
     <row r="7" ht="130" customHeight="1" spans="1:6">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="11" t="s">
         <v>358</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="11" t="s">
         <v>359</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="11" t="s">
         <v>360</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="D7" s="11" t="s">
         <v>361</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="E7" s="11" t="s">
         <v>362</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="F7" s="11" t="s">
         <v>363</v>
       </c>
     </row>
     <row r="8" ht="130" customHeight="1" spans="1:6">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="11" t="s">
         <v>364</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="11" t="s">
         <v>365</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="11" t="s">
         <v>366</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="11" t="s">
         <v>343</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="E8" s="11" t="s">
         <v>367</v>
       </c>
-      <c r="F8" s="8" t="s">
+      <c r="F8" s="11" t="s">
         <v>368</v>
       </c>
     </row>
     <row r="9" ht="130" customHeight="1" spans="1:6">
-      <c r="A9" s="8" t="s">
+      <c r="A9" s="11" t="s">
         <v>369</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="11" t="s">
         <v>370</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="11" t="s">
         <v>371</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="D9" s="11" t="s">
         <v>372</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="E9" s="11" t="s">
         <v>373</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="F9" s="11" t="s">
         <v>374</v>
       </c>
     </row>
     <row r="10" ht="130" customHeight="1" spans="1:6">
-      <c r="A10" s="8" t="s">
+      <c r="A10" s="11" t="s">
         <v>375</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="11" t="s">
         <v>376</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="C10" s="11" t="s">
         <v>377</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="D10" s="11" t="s">
         <v>378</v>
       </c>
-      <c r="E10" s="8" t="s">
+      <c r="E10" s="11" t="s">
         <v>379</v>
       </c>
-      <c r="F10" s="8" t="s">
+      <c r="F10" s="11" t="s">
         <v>380</v>
       </c>
     </row>
     <row r="11" ht="130" customHeight="1" spans="1:6">
-      <c r="A11" s="8" t="s">
+      <c r="A11" s="11" t="s">
         <v>381</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="11" t="s">
         <v>382</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="11" t="s">
         <v>383</v>
       </c>
-      <c r="D11" s="8" t="s">
+      <c r="D11" s="11" t="s">
         <v>378</v>
       </c>
-      <c r="E11" s="8" t="s">
+      <c r="E11" s="11" t="s">
         <v>384</v>
       </c>
-      <c r="F11" s="8" t="s">
+      <c r="F11" s="11" t="s">
         <v>385</v>
       </c>
     </row>
     <row r="12" ht="130" customHeight="1" spans="1:6">
-      <c r="A12" s="8" t="s">
+      <c r="A12" s="11" t="s">
         <v>386</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="11" t="s">
         <v>387</v>
       </c>
-      <c r="C12" s="8" t="s">
+      <c r="C12" s="11" t="s">
         <v>388</v>
       </c>
-      <c r="D12" s="8" t="s">
+      <c r="D12" s="11" t="s">
         <v>378</v>
       </c>
-      <c r="E12" s="8" t="s">
+      <c r="E12" s="11" t="s">
         <v>389</v>
       </c>
-      <c r="F12" s="8" t="s">
+      <c r="F12" s="11" t="s">
         <v>390</v>
       </c>
     </row>
     <row r="13" ht="130" customHeight="1" spans="1:6">
-      <c r="A13" s="8" t="s">
+      <c r="A13" s="11" t="s">
         <v>391</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="11" t="s">
         <v>392</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="C13" s="11" t="s">
         <v>393</v>
       </c>
-      <c r="D13" s="8" t="s">
+      <c r="D13" s="11" t="s">
         <v>378</v>
       </c>
-      <c r="E13" s="8" t="s">
+      <c r="E13" s="11" t="s">
         <v>394</v>
       </c>
-      <c r="F13" s="8" t="s">
+      <c r="F13" s="11" t="s">
         <v>395</v>
       </c>
     </row>
     <row r="14" ht="130" customHeight="1" spans="1:6">
-      <c r="A14" s="8" t="s">
+      <c r="A14" s="11" t="s">
         <v>396</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="B14" s="11" t="s">
         <v>397</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="C14" s="11" t="s">
         <v>398</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="D14" s="11" t="s">
         <v>378</v>
       </c>
-      <c r="E14" s="8" t="s">
+      <c r="E14" s="11" t="s">
         <v>399</v>
       </c>
-      <c r="F14" s="8" t="s">
+      <c r="F14" s="11" t="s">
         <v>400</v>
       </c>
     </row>
@@ -9474,242 +9522,242 @@
       </c>
     </row>
     <row r="2" ht="333" customHeight="1" spans="1:6">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="10" t="s">
         <v>401</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="10" t="s">
         <v>402</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="10" t="s">
         <v>403</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="D2" s="10" t="s">
         <v>404</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="E2" s="10" t="s">
         <v>405</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="F2" s="10" t="s">
         <v>406</v>
       </c>
     </row>
     <row r="3" ht="193" customHeight="1" spans="1:6">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="10" t="s">
         <v>407</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="10" t="s">
         <v>408</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="10" t="s">
         <v>409</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="10" t="s">
         <v>410</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="10" t="s">
         <v>411</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F3" s="10" t="s">
         <v>412</v>
       </c>
     </row>
     <row r="4" ht="130" customHeight="1" spans="1:6">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="10" t="s">
         <v>413</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="10" t="s">
         <v>414</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="10" t="s">
         <v>415</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="10" t="s">
         <v>416</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4" s="10" t="s">
         <v>417</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F4" s="10" t="s">
         <v>418</v>
       </c>
     </row>
     <row r="5" ht="130" customHeight="1" spans="1:6">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="10" t="s">
         <v>419</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="10" t="s">
         <v>420</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="10" t="s">
         <v>421</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="10" t="s">
         <v>422</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="10" t="s">
         <v>423</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="F5" s="10" t="s">
         <v>424</v>
       </c>
     </row>
     <row r="6" ht="130" customHeight="1" spans="1:6">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="10" t="s">
         <v>425</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="10" t="s">
         <v>426</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="10" t="s">
         <v>427</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="10" t="s">
         <v>428</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="10" t="s">
         <v>429</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="F6" s="10" t="s">
         <v>430</v>
       </c>
     </row>
     <row r="7" ht="130" customHeight="1" spans="1:6">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="10" t="s">
         <v>431</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="10" t="s">
         <v>432</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="10" t="s">
         <v>433</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="10" t="s">
         <v>434</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="10" t="s">
         <v>435</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="F7" s="10" t="s">
         <v>436</v>
       </c>
     </row>
     <row r="8" ht="130" customHeight="1" spans="1:6">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="10" t="s">
         <v>437</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="10" t="s">
         <v>438</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="10" t="s">
         <v>439</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="10" t="s">
         <v>440</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="10" t="s">
         <v>441</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="10" t="s">
         <v>442</v>
       </c>
     </row>
     <row r="9" ht="130" customHeight="1" spans="1:6">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="10" t="s">
         <v>443</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="10" t="s">
         <v>444</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="10" t="s">
         <v>445</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="10" t="s">
         <v>440</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="10" t="s">
         <v>446</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="10" t="s">
         <v>447</v>
       </c>
     </row>
     <row r="10" ht="130" customHeight="1" spans="1:6">
-      <c r="A10" s="7" t="s">
+      <c r="A10" s="10" t="s">
         <v>448</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="10" t="s">
         <v>449</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="10" t="s">
         <v>450</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="10" t="s">
         <v>440</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E10" s="10" t="s">
         <v>451</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="F10" s="10" t="s">
         <v>452</v>
       </c>
     </row>
     <row r="11" ht="130" customHeight="1" spans="1:6">
-      <c r="A11" s="7" t="s">
+      <c r="A11" s="10" t="s">
         <v>453</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="10" t="s">
         <v>454</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="10" t="s">
         <v>455</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="D11" s="10" t="s">
         <v>440</v>
       </c>
-      <c r="E11" s="7" t="s">
+      <c r="E11" s="10" t="s">
         <v>456</v>
       </c>
-      <c r="F11" s="7" t="s">
+      <c r="F11" s="10" t="s">
         <v>457</v>
       </c>
     </row>
     <row r="12" ht="130" customHeight="1" spans="1:6">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="10" t="s">
         <v>458</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="10" t="s">
         <v>459</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="10" t="s">
         <v>460</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="10" t="s">
         <v>440</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="E12" s="10" t="s">
         <v>461</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="F12" s="10" t="s">
         <v>462</v>
       </c>
     </row>
     <row r="13" ht="130" customHeight="1" spans="1:6">
-      <c r="A13" s="7" t="s">
+      <c r="A13" s="10" t="s">
         <v>463</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="10" t="s">
         <v>464</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="C13" s="10" t="s">
         <v>465</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="D13" s="10" t="s">
         <v>466</v>
       </c>
-      <c r="E13" s="7" t="s">
+      <c r="E13" s="10" t="s">
         <v>467</v>
       </c>
-      <c r="F13" s="7" t="s">
+      <c r="F13" s="10" t="s">
         <v>468</v>
       </c>
     </row>
@@ -9754,262 +9802,262 @@
       </c>
     </row>
     <row r="2" ht="301" customHeight="1" spans="1:6">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="7" t="s">
         <v>469</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="7" t="s">
         <v>470</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="7" t="s">
         <v>471</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="7" t="s">
         <v>472</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="7" t="s">
         <v>473</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="7" t="s">
         <v>474</v>
       </c>
     </row>
     <row r="3" ht="258" customHeight="1" spans="1:6">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="7" t="s">
         <v>475</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="7" t="s">
         <v>476</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="7" t="s">
         <v>477</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="7" t="s">
         <v>472</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="7" t="s">
         <v>478</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="7" t="s">
         <v>479</v>
       </c>
     </row>
     <row r="4" ht="297" customHeight="1" spans="1:6">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="7" t="s">
         <v>480</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="7" t="s">
         <v>481</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="7" t="s">
         <v>482</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="7" t="s">
         <v>472</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="7" t="s">
         <v>483</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="7" t="s">
         <v>484</v>
       </c>
     </row>
     <row r="5" ht="311" customHeight="1" spans="1:6">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="7" t="s">
         <v>485</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="7" t="s">
         <v>486</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="7" t="s">
         <v>487</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="7" t="s">
         <v>472</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" s="7" t="s">
         <v>488</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="F5" s="7" t="s">
         <v>489</v>
       </c>
     </row>
-    <row r="6" ht="316" customHeight="1" spans="1:6">
-      <c r="A6" s="6" t="s">
+    <row r="6" s="6" customFormat="1" ht="316" customHeight="1" spans="1:6">
+      <c r="A6" s="8" t="s">
         <v>490</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="8" t="s">
         <v>491</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="8" t="s">
         <v>492</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="8" t="s">
         <v>472</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="8" t="s">
         <v>493</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="F6" s="8" t="s">
         <v>494</v>
       </c>
     </row>
     <row r="7" ht="313" customHeight="1" spans="1:6">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="7" t="s">
         <v>495</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="7" t="s">
         <v>496</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="7" t="s">
         <v>497</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="7" t="s">
         <v>498</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="7" t="s">
         <v>499</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="F7" s="7" t="s">
         <v>500</v>
       </c>
     </row>
     <row r="8" ht="197" customHeight="1" spans="1:6">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="7" t="s">
         <v>501</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="9" t="s">
         <v>502</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="7" t="s">
         <v>503</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" s="7" t="s">
         <v>504</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="E8" s="7" t="s">
         <v>505</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="F8" s="7" t="s">
         <v>506</v>
       </c>
     </row>
     <row r="9" ht="312" customHeight="1" spans="1:6">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="7" t="s">
         <v>507</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="7" t="s">
         <v>508</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="7" t="s">
         <v>509</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="7" t="s">
         <v>472</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="E9" s="7" t="s">
         <v>510</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="F9" s="7" t="s">
         <v>511</v>
       </c>
     </row>
     <row r="10" ht="247" customHeight="1" spans="1:6">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="7" t="s">
         <v>512</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="7" t="s">
         <v>513</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="7" t="s">
         <v>514</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="D10" s="7" t="s">
         <v>472</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="E10" s="7" t="s">
         <v>515</v>
       </c>
-      <c r="F10" s="6" t="s">
+      <c r="F10" s="7" t="s">
         <v>516</v>
       </c>
     </row>
     <row r="11" ht="348" customHeight="1" spans="1:6">
-      <c r="A11" s="6" t="s">
+      <c r="A11" s="7" t="s">
         <v>517</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="7" t="s">
         <v>518</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="7" t="s">
         <v>519</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="D11" s="7" t="s">
         <v>520</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="E11" s="7" t="s">
         <v>521</v>
       </c>
-      <c r="F11" s="6" t="s">
+      <c r="F11" s="7" t="s">
         <v>522</v>
       </c>
     </row>
     <row r="12" ht="257" customHeight="1" spans="1:6">
-      <c r="A12" s="6" t="s">
+      <c r="A12" s="7" t="s">
         <v>523</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="7" t="s">
         <v>524</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C12" s="7" t="s">
         <v>525</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="D12" s="7" t="s">
         <v>526</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="E12" s="7" t="s">
         <v>527</v>
       </c>
-      <c r="F12" s="6" t="s">
+      <c r="F12" s="7" t="s">
         <v>528</v>
       </c>
     </row>
     <row r="13" ht="343" customHeight="1" spans="1:6">
-      <c r="A13" s="6" t="s">
+      <c r="A13" s="7" t="s">
         <v>529</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="7" t="s">
         <v>530</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="7" t="s">
         <v>531</v>
       </c>
-      <c r="D13" s="6" t="s">
+      <c r="D13" s="7" t="s">
         <v>472</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="E13" s="7" t="s">
         <v>532</v>
       </c>
-      <c r="F13" s="6" t="s">
+      <c r="F13" s="7" t="s">
         <v>533</v>
       </c>
     </row>
     <row r="14" ht="341" customHeight="1" spans="1:6">
-      <c r="A14" s="6" t="s">
+      <c r="A14" s="7" t="s">
         <v>534</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="7" t="s">
         <v>535</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" s="7" t="s">
         <v>536</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="D14" s="7" t="s">
         <v>537</v>
       </c>
-      <c r="E14" s="6" t="s">
+      <c r="E14" s="7" t="s">
         <v>538</v>
       </c>
-      <c r="F14" s="6" t="s">
+      <c r="F14" s="7" t="s">
         <v>539</v>
       </c>
     </row>

</xml_diff>

<commit_message>
配置用户级互通后，执行docker exec bob-net-test ping -c 3 172.26.0.2不通修复
</commit_message>
<xml_diff>
--- a/docker-authz-proxy-testcases-v3.xlsx
+++ b/docker-authz-proxy-testcases-v3.xlsx
@@ -3492,10 +3492,10 @@
    $ su - alice -c 'docker run -d --name alice-web nginx:alpine'
 2. bob 尝试停止 alice 容器：
    $ su - bob -c 'docker stop alice-web'
-   # 预期：Error response from daemon: container 'alice-web' is not owned by 'bob'(uid=1002)
+   # 预期：Error response from daemon: No such container: alice-web
 3. bob 尝试删除 alice 容器：
    $ su - bob -c 'docker rm alice-web'
-   # 预期：Error response from daemon: container 'alice-web' is not owned by 'bob'(uid=1002)
+   # 预期：Error response from daemon: No such container: alice-web
 4. bob 尝试 exec 进入 alice 容器：
    $ su - bob -c 'docker exec alice-web ls'
    # 预期：Error: No such container: alice-web
@@ -3530,7 +3530,7 @@
    # 预期：不显示 alice-net 或其带前缀版本
 3. bob 尝试连接 alice 网络：
    $ su - bob -c 'docker network connect alice-net $(docker run -d nginx:alpine)'
-   # 预期：Error: network alice-net not found
+   # 预期：Error response from daemon: network alice-net not found
 4. 验证 alice 网络真实名称（root 视角）：
    # docker network ls | grep alice
    # 预期：显示 alice_u1004_alice-net
@@ -3592,11 +3592,7 @@
        --label system.authz.owner.uid=1004 \
        --name bob-fake nginx:alpine'
 2. 检查实际标签（代理应覆盖）：
-   # docker inspect user-1003-bob-fake | python3 -c "
-     import json,sys; d=json.load(sys.stdin)[0]
-     labels = d['Config']['Labels']
-     print('owner.uid:', labels.get('system.authz.owner.uid'))
-     print('期望: 1003 (bob 的真实 uid)')"
+   # docker inspect bob-fake | python3 -c 'import json,sys; d=json.load(sys.stdin)[0]; labels=d["Config"]["Labels"]; print("owner.uid:", labels.get("system.authz.owner.uid")); print("期望: 1003 (bob  的真实 uid)")'
 3. 验证 alice 无法看到该容器：
    $ su - alice -c 'docker ps -a | grep bob-fake'
    # 预期：无输出
@@ -5859,7 +5855,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="50">
+  <fills count="48">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -5898,19 +5894,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFE2EFDA"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -6300,7 +6284,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -6324,16 +6308,16 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="20" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="18" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="21" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="19" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="21" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="19" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="22" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="20" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -6342,85 +6326,85 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="43" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="44" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="45" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="43" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="46" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="44" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="47" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="45" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="48" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="46" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="49" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="47" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -6441,14 +6425,20 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -6463,29 +6453,23 @@
     <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>

</xml_diff>